<commit_message>
Update algorithm for phy_weight_method
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NHANES11.xlsx
+++ b/baseline/data_processing_elements-NHANES11.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A153B386-4332-4473-9E30-1ED3AC4B2EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAEBE6DB-3915-467D-BD36-8DAB0DA5E676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3161BE6F-2E10-4AFE-B2DF-B65F0CC4B714}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2099" uniqueCount="884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2100" uniqueCount="885">
   <si>
     <t>index</t>
   </si>
@@ -2905,11 +2905,6 @@
   </si>
   <si>
     <t>MCQ160A</t>
-  </si>
-  <si>
-    <t>case_when(
-BMIWT != 4 &amp; ! is.na(BMIWT) ~ 2L; 
-ELSE ~ NA_integer_)</t>
   </si>
   <si>
     <t>DXDTOPF</t>
@@ -3630,6 +3625,15 @@
   <si>
     <t xml:space="preserve">Non-drinkers were coded as 0. The study-specific information was based on responses about alcohol use in the past 12 months. Mean grams of alcohol per standard drink in the United States (14g) was used for calculations. 
 </t>
+  </si>
+  <si>
+    <t>Additional updates following crosschecks.</t>
+  </si>
+  <si>
+    <t>case_when(
+BMIWT == 4 ~ NA_integer_; 
+!is.na(BMIWT) ~ 2L; 
+ELSE ~ NA_integer_)</t>
   </si>
 </sst>
 </file>
@@ -4164,7 +4168,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>10</v>
@@ -4194,10 +4198,10 @@
         <v>17</v>
       </c>
       <c r="U1" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="V1" s="10" t="s">
         <v>770</v>
-      </c>
-      <c r="V1" s="10" t="s">
-        <v>771</v>
       </c>
       <c r="W1" s="10" t="s">
         <v>18</v>
@@ -4391,7 +4395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:32" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -4420,7 +4424,7 @@
         <v>472</v>
       </c>
       <c r="U6" s="12" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="V6" s="3" t="s">
         <v>474</v>
@@ -4491,7 +4495,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -4535,7 +4539,7 @@
         <v>487</v>
       </c>
       <c r="U8" s="12" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="V8" s="3" t="s">
         <v>468</v>
@@ -4597,7 +4601,7 @@
         <v>494</v>
       </c>
       <c r="U9" s="12" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="V9" s="3" t="s">
         <v>468</v>
@@ -4609,13 +4613,13 @@
         <v>496</v>
       </c>
       <c r="Y9" s="12" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="Z9" s="4" t="s">
         <v>497</v>
       </c>
       <c r="AB9" s="4" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="10" spans="1:32" ht="409.5" x14ac:dyDescent="0.25">
@@ -4671,13 +4675,13 @@
         <v>496</v>
       </c>
       <c r="Y10" s="12" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="Z10" s="4" t="s">
         <v>497</v>
       </c>
       <c r="AB10" s="4" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="11" spans="1:32" ht="120" x14ac:dyDescent="0.25">
@@ -5164,7 +5168,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="135" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -5211,7 +5215,7 @@
         <v>501</v>
       </c>
       <c r="U19" s="12" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="V19" s="3" t="s">
         <v>468</v>
@@ -5270,7 +5274,7 @@
         <v>513</v>
       </c>
       <c r="U20" s="12" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="V20" s="3" t="s">
         <v>468</v>
@@ -5282,13 +5286,13 @@
         <v>482</v>
       </c>
       <c r="Y20" s="12" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="Z20" s="12" t="s">
         <v>514</v>
       </c>
       <c r="AB20" s="4" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="21" spans="1:28" ht="330" x14ac:dyDescent="0.25">
@@ -5317,7 +5321,7 @@
         <v>427</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="M21" s="4" t="s">
         <v>518</v>
@@ -5338,7 +5342,7 @@
         <v>521</v>
       </c>
       <c r="U21" s="4" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="V21" s="3" t="s">
         <v>468</v>
@@ -5350,13 +5354,13 @@
         <v>496</v>
       </c>
       <c r="Y21" s="12" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="Z21" s="4" t="s">
         <v>516</v>
       </c>
       <c r="AB21" s="4" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="22" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -5382,7 +5386,7 @@
         <v>353</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="M22" s="4" t="s">
         <v>517</v>
@@ -5403,7 +5407,7 @@
         <v>524</v>
       </c>
       <c r="U22" s="12" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="V22" s="3" t="s">
         <v>468</v>
@@ -5415,16 +5419,16 @@
         <v>496</v>
       </c>
       <c r="Y22" s="12" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="Z22" s="4" t="s">
         <v>701</v>
       </c>
       <c r="AB22" s="4" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="23" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" ht="405" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -5459,7 +5463,7 @@
         <v>698</v>
       </c>
       <c r="U23" s="12" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="V23" s="3" t="s">
         <v>468</v>
@@ -5521,7 +5525,7 @@
         <v>528</v>
       </c>
       <c r="U24" s="12" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="V24" s="3" t="s">
         <v>468</v>
@@ -5533,13 +5537,13 @@
         <v>496</v>
       </c>
       <c r="Y24" s="12" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="Z24" s="4" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="AB24" s="4" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="25" spans="1:28" ht="135" x14ac:dyDescent="0.25">
@@ -5595,10 +5599,10 @@
         <v>482</v>
       </c>
       <c r="Y25" s="12" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="AB25" s="4" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="26" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -5668,7 +5672,7 @@
         <v>389</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="M27" s="4" t="s">
         <v>533</v>
@@ -5689,7 +5693,7 @@
         <v>702</v>
       </c>
       <c r="U27" s="12" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="V27" s="3" t="s">
         <v>468</v>
@@ -5730,7 +5734,7 @@
         <v>431</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="M28" s="4" t="s">
         <v>533</v>
@@ -5792,7 +5796,7 @@
         <v>389</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="M29" s="4" t="s">
         <v>537</v>
@@ -5813,7 +5817,7 @@
         <v>705</v>
       </c>
       <c r="U29" s="12" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="V29" s="3" t="s">
         <v>468</v>
@@ -5854,7 +5858,7 @@
         <v>431</v>
       </c>
       <c r="L30" s="4" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="M30" s="4" t="s">
         <v>537</v>
@@ -5883,11 +5887,14 @@
       <c r="X30" s="3" t="s">
         <v>496</v>
       </c>
-      <c r="Y30" s="4" t="s">
-        <v>736</v>
+      <c r="Y30" s="12" t="s">
+        <v>884</v>
       </c>
       <c r="Z30" s="4" t="s">
         <v>704</v>
+      </c>
+      <c r="AB30" s="12" t="s">
+        <v>883</v>
       </c>
     </row>
     <row r="31" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -5972,7 +5979,7 @@
         <v>389</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="M32" s="4" t="s">
         <v>541</v>
@@ -6028,7 +6035,7 @@
         <v>431</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="M33" s="4" t="s">
         <v>541</v>
@@ -6081,7 +6088,7 @@
         <v>357</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="M34" s="4" t="s">
         <v>544</v>
@@ -6102,7 +6109,7 @@
         <v>547</v>
       </c>
       <c r="U34" s="12" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="V34" s="3" t="s">
         <v>468</v>
@@ -6137,7 +6144,7 @@
         <v>347</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="M35" s="4" t="s">
         <v>544</v>
@@ -6170,7 +6177,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="345" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:28" ht="330" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -6217,7 +6224,7 @@
         <v>552</v>
       </c>
       <c r="U36" s="12" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="V36" s="3" t="s">
         <v>468</v>
@@ -6229,17 +6236,17 @@
         <v>554</v>
       </c>
       <c r="Y36" s="12" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="Z36" s="4" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="AA36" s="4"/>
       <c r="AB36" s="4" t="s">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="37" spans="1:28" ht="345" x14ac:dyDescent="0.25">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" ht="330" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -6286,7 +6293,7 @@
         <v>557</v>
       </c>
       <c r="U37" s="12" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="V37" s="3" t="s">
         <v>468</v>
@@ -6298,13 +6305,13 @@
         <v>554</v>
       </c>
       <c r="Y37" s="12" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="Z37" s="4" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="AB37" s="4" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
     <row r="38" spans="1:28" ht="105" x14ac:dyDescent="0.25">
@@ -6333,7 +6340,7 @@
         <v>390</v>
       </c>
       <c r="L38" s="4" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="M38" s="4" t="s">
         <v>558</v>
@@ -6354,7 +6361,7 @@
         <v>560</v>
       </c>
       <c r="U38" s="12" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="V38" s="3" t="s">
         <v>468</v>
@@ -6436,7 +6443,7 @@
         <v>432</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="M40" s="4" t="s">
         <v>561</v>
@@ -6457,7 +6464,7 @@
         <v>565</v>
       </c>
       <c r="U40" s="12" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V40" s="3" t="s">
         <v>468</v>
@@ -6469,7 +6476,7 @@
         <v>496</v>
       </c>
       <c r="Y40" s="4" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="Z40" s="4" t="s">
         <v>566</v>
@@ -6498,7 +6505,7 @@
         <v>361</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="M41" s="4" t="s">
         <v>567</v>
@@ -6534,7 +6541,7 @@
         <v>489</v>
       </c>
       <c r="AB41" s="4" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="42" spans="1:28" ht="90" x14ac:dyDescent="0.25">
@@ -6560,7 +6567,7 @@
         <v>362</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="M42" s="4" t="s">
         <v>572</v>
@@ -6593,13 +6600,13 @@
         <v>496</v>
       </c>
       <c r="Y42" s="12" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="Z42" s="4" t="s">
         <v>575</v>
       </c>
       <c r="AB42" s="4" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="43" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -6625,7 +6632,7 @@
         <v>363</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="M43" s="4" t="s">
         <v>578</v>
@@ -6684,7 +6691,7 @@
         <v>363</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="M44" s="4" t="s">
         <v>579</v>
@@ -6758,7 +6765,7 @@
         <v>474</v>
       </c>
       <c r="Z45" s="4" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="46" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -6787,7 +6794,7 @@
         <v>392</v>
       </c>
       <c r="L46" s="4" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="M46" s="4" t="s">
         <v>583</v>
@@ -6811,7 +6818,7 @@
         <v>363</v>
       </c>
       <c r="U46" s="12" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="V46" s="3" t="s">
         <v>468</v>
@@ -6852,7 +6859,7 @@
         <v>363</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="M47" s="4" t="s">
         <v>588</v>
@@ -7128,7 +7135,7 @@
         <v>711</v>
       </c>
       <c r="U53" s="12" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="V53" s="3" t="s">
         <v>468</v>
@@ -7140,13 +7147,13 @@
         <v>496</v>
       </c>
       <c r="Y53" s="4" t="s">
+        <v>777</v>
+      </c>
+      <c r="Z53" s="4" t="s">
         <v>778</v>
       </c>
-      <c r="Z53" s="4" t="s">
-        <v>779</v>
-      </c>
       <c r="AB53" s="4" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="54" spans="1:28" ht="225" x14ac:dyDescent="0.25">
@@ -7193,7 +7200,7 @@
         <v>594</v>
       </c>
       <c r="U54" s="12" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="V54" s="3" t="s">
         <v>468</v>
@@ -7205,10 +7212,10 @@
         <v>496</v>
       </c>
       <c r="Y54" s="12" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="Z54" s="12" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="55" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -7234,7 +7241,7 @@
         <v>434</v>
       </c>
       <c r="L55" s="4" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="M55" s="4" t="s">
         <v>598</v>
@@ -7261,7 +7268,7 @@
         <v>717</v>
       </c>
       <c r="Y55" s="4" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="Z55" s="4" t="s">
         <v>718</v>
@@ -7293,7 +7300,7 @@
         <v>435</v>
       </c>
       <c r="L56" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="M56" s="4" t="s">
         <v>604</v>
@@ -7311,7 +7318,7 @@
         <v>607</v>
       </c>
       <c r="U56" s="12" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="V56" s="3" t="s">
         <v>468</v>
@@ -7326,7 +7333,7 @@
         <v>608</v>
       </c>
       <c r="Z56" s="4" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="57" spans="1:28" ht="120" x14ac:dyDescent="0.25">
@@ -7352,7 +7359,7 @@
         <v>436</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="M57" s="4" t="s">
         <v>601</v>
@@ -7370,7 +7377,7 @@
         <v>609</v>
       </c>
       <c r="U57" s="12" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="V57" s="3" t="s">
         <v>468</v>
@@ -7411,10 +7418,10 @@
         <v>398</v>
       </c>
       <c r="L58" s="4" t="s">
+        <v>876</v>
+      </c>
+      <c r="M58" s="4" t="s">
         <v>877</v>
-      </c>
-      <c r="M58" s="4" t="s">
-        <v>878</v>
       </c>
       <c r="N58" s="3" t="s">
         <v>602</v>
@@ -7426,10 +7433,10 @@
         <v>611</v>
       </c>
       <c r="S58" s="4" t="s">
+        <v>878</v>
+      </c>
+      <c r="U58" s="12" t="s">
         <v>879</v>
-      </c>
-      <c r="U58" s="12" t="s">
-        <v>880</v>
       </c>
       <c r="V58" s="3" t="s">
         <v>468</v>
@@ -7441,10 +7448,10 @@
         <v>496</v>
       </c>
       <c r="Y58" s="12" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="Z58" s="4" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="59" spans="1:28" ht="75" x14ac:dyDescent="0.25">
@@ -7470,7 +7477,7 @@
         <v>353</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="M59" s="4" t="s">
         <v>612</v>
@@ -7485,7 +7492,7 @@
         <v>614</v>
       </c>
       <c r="U59" s="12" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="V59" s="3" t="s">
         <v>468</v>
@@ -7526,7 +7533,7 @@
         <v>437</v>
       </c>
       <c r="L60" s="3" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="M60" s="4" t="s">
         <v>612</v>
@@ -7553,7 +7560,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="61" spans="1:28" ht="135" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -7635,7 +7642,7 @@
         <v>439</v>
       </c>
       <c r="L62" s="3" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="M62" s="4" t="s">
         <v>622</v>
@@ -7653,7 +7660,7 @@
         <v>627</v>
       </c>
       <c r="U62" s="12" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="V62" s="3" t="s">
         <v>468</v>
@@ -7770,7 +7777,7 @@
         <v>440</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="M65" s="4" t="s">
         <v>630</v>
@@ -7788,7 +7795,7 @@
         <v>627</v>
       </c>
       <c r="U65" s="12" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="V65" s="3" t="s">
         <v>468</v>
@@ -7832,7 +7839,7 @@
         <v>439</v>
       </c>
       <c r="L66" s="3" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="M66" s="4" t="s">
         <v>630</v>
@@ -7850,7 +7857,7 @@
         <v>627</v>
       </c>
       <c r="U66" s="12" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="V66" s="3" t="s">
         <v>474</v>
@@ -7906,7 +7913,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="68" spans="1:28" ht="225" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:28" ht="210" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>67</v>
       </c>
@@ -7914,7 +7921,7 @@
         <v>465</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>214</v>
@@ -7932,7 +7939,7 @@
         <v>399</v>
       </c>
       <c r="L68" s="3" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="M68" s="4" t="s">
         <v>632</v>
@@ -7960,16 +7967,16 @@
         <v>496</v>
       </c>
       <c r="Y68" s="12" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="Z68" s="12" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="AB68" s="4" t="s">
-        <v>833</v>
-      </c>
-    </row>
-    <row r="69" spans="1:28" ht="225" x14ac:dyDescent="0.25">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="69" spans="1:28" ht="210" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -7992,7 +7999,7 @@
         <v>441</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="M69" s="4" t="s">
         <v>632</v>
@@ -8023,13 +8030,13 @@
         <v>496</v>
       </c>
       <c r="Y69" s="12" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="Z69" s="12" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="AB69" s="4" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="70" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -8137,7 +8144,7 @@
         <v>472</v>
       </c>
       <c r="U72" s="12" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="V72" s="3" t="s">
         <v>474</v>
@@ -8155,7 +8162,7 @@
         <v>637</v>
       </c>
       <c r="AB72" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="73" spans="1:28" ht="210" x14ac:dyDescent="0.25">
@@ -8202,7 +8209,7 @@
         <v>645</v>
       </c>
       <c r="U73" s="12" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="V73" s="3" t="s">
         <v>468</v>
@@ -8220,7 +8227,7 @@
         <v>720</v>
       </c>
       <c r="AB73" s="4" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="74" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -8276,10 +8283,10 @@
         <v>496</v>
       </c>
       <c r="Y74" s="4" t="s">
+        <v>779</v>
+      </c>
+      <c r="Z74" s="4" t="s">
         <v>780</v>
-      </c>
-      <c r="Z74" s="4" t="s">
-        <v>781</v>
       </c>
     </row>
     <row r="75" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -8381,7 +8388,7 @@
         <v>444</v>
       </c>
       <c r="L77" s="3" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="M77" s="4" t="s">
         <v>647</v>
@@ -8458,7 +8465,7 @@
         <v>641</v>
       </c>
       <c r="U78" s="12" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="V78" s="3" t="s">
         <v>468</v>
@@ -8473,7 +8480,7 @@
         <v>730</v>
       </c>
       <c r="AB78" s="4" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="79" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8526,7 +8533,7 @@
         <v>641</v>
       </c>
       <c r="U79" s="12" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="V79" s="3" t="s">
         <v>468</v>
@@ -8541,7 +8548,7 @@
         <v>672</v>
       </c>
       <c r="AB79" s="4" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="80" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8594,7 +8601,7 @@
         <v>641</v>
       </c>
       <c r="U80" s="12" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="V80" s="3" t="s">
         <v>468</v>
@@ -8868,7 +8875,7 @@
         <v>445</v>
       </c>
       <c r="L85" s="3" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="M85" s="4" t="s">
         <v>662</v>
@@ -8930,16 +8937,16 @@
         <v>445</v>
       </c>
       <c r="L86" s="4" t="s">
+        <v>763</v>
+      </c>
+      <c r="M86" s="4" t="s">
         <v>764</v>
-      </c>
-      <c r="M86" s="4" t="s">
-        <v>765</v>
       </c>
       <c r="N86" s="3" t="s">
         <v>663</v>
       </c>
       <c r="O86" s="4" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="P86" s="4" t="s">
         <v>665</v>
@@ -8951,7 +8958,7 @@
         <v>641</v>
       </c>
       <c r="U86" s="12" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="V86" s="3" t="s">
         <v>468</v>
@@ -8963,10 +8970,10 @@
         <v>496</v>
       </c>
       <c r="Y86" s="4" t="s">
+        <v>766</v>
+      </c>
+      <c r="Z86" s="4" t="s">
         <v>767</v>
-      </c>
-      <c r="Z86" s="4" t="s">
-        <v>768</v>
       </c>
     </row>
     <row r="87" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -9019,7 +9026,7 @@
         <v>641</v>
       </c>
       <c r="U87" s="12" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="V87" s="3" t="s">
         <v>468</v>
@@ -9063,7 +9070,7 @@
         <v>445</v>
       </c>
       <c r="L88" s="3" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="M88" s="4" t="s">
         <v>673</v>
@@ -9160,7 +9167,7 @@
         <v>445</v>
       </c>
       <c r="L90" s="3" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="M90" s="4" t="s">
         <v>678</v>
@@ -9219,25 +9226,25 @@
         <v>445</v>
       </c>
       <c r="L91" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M91" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M91" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N91" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O91" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P91" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P91" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R91" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S91" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V91" s="3" t="s">
         <v>468</v>
@@ -9249,13 +9256,13 @@
         <v>496</v>
       </c>
       <c r="Y91" s="12" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="Z91" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB91" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="92" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9284,25 +9291,25 @@
         <v>445</v>
       </c>
       <c r="L92" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M92" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M92" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N92" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O92" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P92" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P92" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R92" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S92" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V92" s="3" t="s">
         <v>468</v>
@@ -9314,13 +9321,13 @@
         <v>496</v>
       </c>
       <c r="Y92" s="12" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="Z92" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB92" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="93" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9349,25 +9356,25 @@
         <v>445</v>
       </c>
       <c r="L93" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M93" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M93" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N93" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O93" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P93" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P93" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R93" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S93" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V93" s="3" t="s">
         <v>468</v>
@@ -9379,13 +9386,13 @@
         <v>496</v>
       </c>
       <c r="Y93" s="12" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="Z93" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB93" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="94" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9414,25 +9421,25 @@
         <v>445</v>
       </c>
       <c r="L94" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M94" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M94" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N94" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O94" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P94" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P94" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R94" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S94" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V94" s="3" t="s">
         <v>468</v>
@@ -9444,13 +9451,13 @@
         <v>496</v>
       </c>
       <c r="Y94" s="12" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="Z94" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB94" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="95" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9479,25 +9486,25 @@
         <v>445</v>
       </c>
       <c r="L95" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M95" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M95" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N95" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O95" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P95" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P95" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R95" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S95" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V95" s="3" t="s">
         <v>468</v>
@@ -9509,13 +9516,13 @@
         <v>496</v>
       </c>
       <c r="Y95" s="12" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="Z95" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB95" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="96" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9544,25 +9551,25 @@
         <v>445</v>
       </c>
       <c r="L96" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M96" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M96" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N96" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O96" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P96" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P96" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R96" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S96" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V96" s="3" t="s">
         <v>468</v>
@@ -9574,13 +9581,13 @@
         <v>496</v>
       </c>
       <c r="Y96" s="12" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="Z96" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB96" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="97" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9609,25 +9616,25 @@
         <v>445</v>
       </c>
       <c r="L97" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M97" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M97" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N97" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O97" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P97" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P97" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R97" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S97" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V97" s="3" t="s">
         <v>468</v>
@@ -9639,13 +9646,13 @@
         <v>496</v>
       </c>
       <c r="Y97" s="12" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="Z97" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB97" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="98" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9674,25 +9681,25 @@
         <v>445</v>
       </c>
       <c r="L98" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M98" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M98" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N98" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O98" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P98" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P98" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R98" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S98" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V98" s="3" t="s">
         <v>468</v>
@@ -9704,13 +9711,13 @@
         <v>496</v>
       </c>
       <c r="Y98" s="12" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="Z98" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB98" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="99" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9739,25 +9746,25 @@
         <v>445</v>
       </c>
       <c r="L99" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M99" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M99" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N99" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O99" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P99" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P99" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R99" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S99" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V99" s="3" t="s">
         <v>468</v>
@@ -9769,13 +9776,13 @@
         <v>496</v>
       </c>
       <c r="Y99" s="12" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="Z99" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB99" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="100" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9804,25 +9811,25 @@
         <v>445</v>
       </c>
       <c r="L100" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M100" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M100" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N100" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O100" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P100" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P100" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R100" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S100" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V100" s="3" t="s">
         <v>468</v>
@@ -9834,13 +9841,13 @@
         <v>496</v>
       </c>
       <c r="Y100" s="12" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="Z100" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB100" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="101" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9869,25 +9876,25 @@
         <v>445</v>
       </c>
       <c r="L101" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M101" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M101" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N101" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O101" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P101" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P101" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R101" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S101" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V101" s="3" t="s">
         <v>468</v>
@@ -9899,13 +9906,13 @@
         <v>496</v>
       </c>
       <c r="Y101" s="12" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="Z101" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB101" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="102" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9934,25 +9941,25 @@
         <v>445</v>
       </c>
       <c r="L102" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M102" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M102" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N102" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O102" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P102" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P102" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R102" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S102" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V102" s="3" t="s">
         <v>468</v>
@@ -9964,13 +9971,13 @@
         <v>496</v>
       </c>
       <c r="Y102" s="12" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="Z102" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB102" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="103" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9999,25 +10006,25 @@
         <v>445</v>
       </c>
       <c r="L103" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M103" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M103" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N103" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O103" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P103" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P103" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R103" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S103" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V103" s="3" t="s">
         <v>468</v>
@@ -10029,13 +10036,13 @@
         <v>496</v>
       </c>
       <c r="Y103" s="12" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="Z103" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB103" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="104" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10064,25 +10071,25 @@
         <v>445</v>
       </c>
       <c r="L104" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M104" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M104" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N104" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O104" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P104" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P104" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R104" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S104" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V104" s="3" t="s">
         <v>468</v>
@@ -10094,13 +10101,13 @@
         <v>496</v>
       </c>
       <c r="Y104" s="12" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="Z104" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB104" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="105" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10129,25 +10136,25 @@
         <v>445</v>
       </c>
       <c r="L105" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M105" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M105" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N105" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O105" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P105" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P105" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R105" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S105" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V105" s="3" t="s">
         <v>468</v>
@@ -10159,13 +10166,13 @@
         <v>496</v>
       </c>
       <c r="Y105" s="12" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="Z105" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB105" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="106" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10194,25 +10201,25 @@
         <v>445</v>
       </c>
       <c r="L106" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M106" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M106" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N106" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O106" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P106" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P106" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R106" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S106" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V106" s="3" t="s">
         <v>468</v>
@@ -10224,13 +10231,13 @@
         <v>496</v>
       </c>
       <c r="Y106" s="12" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="Z106" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB106" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="107" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10259,25 +10266,25 @@
         <v>445</v>
       </c>
       <c r="L107" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M107" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M107" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N107" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O107" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P107" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P107" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R107" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S107" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V107" s="3" t="s">
         <v>468</v>
@@ -10289,13 +10296,13 @@
         <v>496</v>
       </c>
       <c r="Y107" s="12" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="Z107" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB107" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="108" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10324,25 +10331,25 @@
         <v>445</v>
       </c>
       <c r="L108" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M108" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M108" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N108" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O108" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P108" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P108" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R108" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S108" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V108" s="3" t="s">
         <v>468</v>
@@ -10354,13 +10361,13 @@
         <v>496</v>
       </c>
       <c r="Y108" s="12" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="Z108" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB108" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="109" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10389,25 +10396,25 @@
         <v>445</v>
       </c>
       <c r="L109" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="M109" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="M109" s="4" t="s">
-        <v>773</v>
       </c>
       <c r="N109" s="3" t="s">
         <v>653</v>
       </c>
       <c r="O109" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="P109" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="P109" s="4" t="s">
-        <v>775</v>
       </c>
       <c r="R109" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S109" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="V109" s="3" t="s">
         <v>468</v>
@@ -10419,13 +10426,13 @@
         <v>496</v>
       </c>
       <c r="Y109" s="12" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="Z109" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AB109" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="110" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -10595,10 +10602,10 @@
         <v>445</v>
       </c>
       <c r="L113" s="12" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="M113" s="12" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="N113" s="3" t="s">
         <v>727</v>
@@ -10607,10 +10614,10 @@
         <v>721</v>
       </c>
       <c r="S113" s="12" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="U113" s="12" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="V113" s="3" t="s">
         <v>468</v>
@@ -10622,13 +10629,13 @@
         <v>496</v>
       </c>
       <c r="Y113" s="12" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="Z113" s="4" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="AB113" s="4" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="114" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -10678,7 +10685,7 @@
         <v>641</v>
       </c>
       <c r="U114" s="12" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="V114" s="3" t="s">
         <v>468</v>
@@ -10722,7 +10729,7 @@
         <v>445</v>
       </c>
       <c r="L115" s="4" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="M115" s="4" t="s">
         <v>685</v>
@@ -10752,10 +10759,10 @@
         <v>496</v>
       </c>
       <c r="Y115" s="4" t="s">
+        <v>784</v>
+      </c>
+      <c r="Z115" s="4" t="s">
         <v>785</v>
-      </c>
-      <c r="Z115" s="4" t="s">
-        <v>786</v>
       </c>
     </row>
     <row r="116" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -10960,7 +10967,7 @@
         <v>496</v>
       </c>
       <c r="Y120" s="4" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="Z120" s="4" t="s">
         <v>722</v>

</xml_diff>